<commit_message>
Add Stag's Leap producer mapping (code: StagsLeap)
- Discount Code Mapping: Stag's Leap / StagsLeap / standalone producer
- Product Mapping: Napa (not cult wine) tier; US / California region

Distinct from the existing Staglin producer. Apostrophe in the producer
name is handled by the _norm apostrophe-stripping on lookup.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3663,6 +3663,23 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Stag's Leap</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>StagsLeap</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Cliff Lede Poetry producer and Vega code under Vega Sicilia
- Cliff Lede Poetry / CliffLede / standalone producer; tier Napa (not
  cult wine); region US / California.
- Vega (Vega Sicilia Valbuena product line) appended to Vega Sicilia's
  codes: Unico, Tempranillo, Vega — inherits Super Second / Spain.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D179"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>Unico, Tempranillo</t>
+          <t>Unico, Tempranillo, Vega</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
@@ -3675,6 +3675,23 @@
         </is>
       </c>
       <c r="C179" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Cliff Lede Poetry</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>CliffLede</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
         <is>
           <t>standalone producer</t>
         </is>

</xml_diff>

<commit_message>
Add 3 producer mappings: LesCarmesHB, Macdonald, Araujo
- Les Carmes Haut-Brion / LesCarmesHB — Super Second Producers,
  France / Bordeaux Left Bank (distinct from Haut Brion First Growth)
- Macdonald / Macdonald — Napa (not cult wine), US / California
- Araujo Estate / Araujo — Napa (not cult wine), US / California
  (distinct from existing Eisele/EISELE and Combo - Araujo + Eisele/
  Altagracia entries; no code collisions)

All three standalone producer offer type.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3697,6 +3697,57 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Les Carmes Haut-Brion</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>LesCarmesHB</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Macdonald</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Macdonald</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Araujo Estate</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Araujo</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Luciano Sandrone producer mapping (code: Sandrone)
Super Second Producers tier; Italy region; standalone producer.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3748,6 +3748,23 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Luciano Sandrone</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Sandrone</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add DallaValle code to Dalla Valle producer
Dalla Valle codes now: Maya, DallaValle. DallaValle covers the
producer's non-Maya offers; inherits Cult Wine Producers - Flagship /
US / California.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Maya</t>
+          <t>Maya, DallaValle</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Split Dalla Valle: Maya is cult wine, other offers are Napa (not cult)
Tier is assigned per producer, so the two codes need separate producer
entries to carry different tiers:
- Dalla Valle Maya / Maya — Cult Wine Producers - Flagship
- Dalla Valle / DallaValle — Napa (not cult wine)
Both US / California, standalone producer.

Past Maya campaigns will now show producer "Dalla Valle Maya".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D184"/>
+  <dimension ref="A1:D185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Maya, DallaValle</t>
+          <t>DallaValle</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
@@ -3762,6 +3762,23 @@
       <c r="C184" t="inlineStr">
         <is>
           <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Dalla Valle Maya</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Maya</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Bonnes-Mares producer mapping (code: BonnesMares)
Blue-chip Burgundy Producer tier; France / Burgundy region; standalone
producer. Separate from the existing Mugnier Bonnes Mares / Mugnier entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D185"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3782,6 +3782,23 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Bonnes-Mares</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>BonnesMares</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>